<commit_message>
added scenarios for add patient
</commit_message>
<xml_diff>
--- a/src/test/resources/DieticianApp_ExcelData.xlsx
+++ b/src/test/resources/DieticianApp_ExcelData.xlsx
@@ -1,37 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/mayaIntellijProjects/SeleniumHackathon/src/test/resources/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E427F7D-B651-FD4E-A4FB-67B17F8C6E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="2328"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="23020" windowHeight="10440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPageContent" sheetId="2" r:id="rId1"/>
+    <sheet name="allergies" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:G22"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
   <si>
     <t>username</t>
   </si>
@@ -103,13 +98,55 @@
   </si>
   <si>
     <t>valid%</t>
+  </si>
+  <si>
+    <t>Allergies</t>
+  </si>
+  <si>
+    <t>Egg</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>Soy</t>
+  </si>
+  <si>
+    <t>Almond</t>
+  </si>
+  <si>
+    <t>Peanuts</t>
+  </si>
+  <si>
+    <t>Walnut</t>
+  </si>
+  <si>
+    <t>Pistachio</t>
+  </si>
+  <si>
+    <t>Sesame</t>
+  </si>
+  <si>
+    <t>Hazelnut</t>
+  </si>
+  <si>
+    <t>Pecan</t>
+  </si>
+  <si>
+    <t>Cashew</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>Values</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,6 +161,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -154,6 +197,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,18 +531,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.09765625" customWidth="1"/>
+    <col min="1" max="1" width="27.1640625" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="25.69921875" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -515,7 +559,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -530,7 +574,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
@@ -545,7 +589,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -560,7 +604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
@@ -575,7 +619,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -590,7 +634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:5" customFormat="1">
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -605,7 +649,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:5" customFormat="1">
+    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -620,7 +664,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:5" customFormat="1">
+    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -641,4 +685,84 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0818B99A-3A20-E546-9E37-758C2D7CCFA5}">
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="16" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added features for new patient
</commit_message>
<xml_diff>
--- a/src/test/resources/DieticianApp_ExcelData.xlsx
+++ b/src/test/resources/DieticianApp_ExcelData.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/mayaIntellijProjects/SeleniumHackathon/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E427F7D-B651-FD4E-A4FB-67B17F8C6E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F822EA0-DF21-AA40-9C1C-946B26F09CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="23020" windowHeight="10440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="23020" windowHeight="10440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPageContent" sheetId="2" r:id="rId1"/>
     <sheet name="allergies" sheetId="3" r:id="rId2"/>
+    <sheet name="foodPreference" sheetId="4" r:id="rId3"/>
+    <sheet name="cuisine" sheetId="5" r:id="rId4"/>
+    <sheet name="requiredFields" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="86">
   <si>
     <t>username</t>
   </si>
@@ -140,6 +143,150 @@
   </si>
   <si>
     <t>Values</t>
+  </si>
+  <si>
+    <t>Vegan</t>
+  </si>
+  <si>
+    <t>NonVeg</t>
+  </si>
+  <si>
+    <t>Eggitarian</t>
+  </si>
+  <si>
+    <t>Jain</t>
+  </si>
+  <si>
+    <t>Indian</t>
+  </si>
+  <si>
+    <t>South Indian</t>
+  </si>
+  <si>
+    <t>Rajasthani</t>
+  </si>
+  <si>
+    <t>Punjabi</t>
+  </si>
+  <si>
+    <t>Bengali</t>
+  </si>
+  <si>
+    <t>Orissa</t>
+  </si>
+  <si>
+    <t>Gujarati</t>
+  </si>
+  <si>
+    <t>Maharashtrian</t>
+  </si>
+  <si>
+    <t>Andhra</t>
+  </si>
+  <si>
+    <t>Kerala</t>
+  </si>
+  <si>
+    <t>Goan</t>
+  </si>
+  <si>
+    <t>Kashmiri</t>
+  </si>
+  <si>
+    <t>Himachali</t>
+  </si>
+  <si>
+    <t>Tamil Nadu</t>
+  </si>
+  <si>
+    <t>Karnataka</t>
+  </si>
+  <si>
+    <t>Sindhi</t>
+  </si>
+  <si>
+    <t>Chhattisgarhi</t>
+  </si>
+  <si>
+    <t>Madhya Pradesh</t>
+  </si>
+  <si>
+    <t>Assamese</t>
+  </si>
+  <si>
+    <t>Manipuri</t>
+  </si>
+  <si>
+    <t>Tripuri</t>
+  </si>
+  <si>
+    <t>Sikkimese</t>
+  </si>
+  <si>
+    <t>Mizo</t>
+  </si>
+  <si>
+    <t>Arunachali</t>
+  </si>
+  <si>
+    <t>Uttarakhand</t>
+  </si>
+  <si>
+    <t>Haryanvi</t>
+  </si>
+  <si>
+    <t>Awadhi</t>
+  </si>
+  <si>
+    <t>Bihari</t>
+  </si>
+  <si>
+    <t>Uttar Pradesh</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>North Indian</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>contactNumber</t>
+  </si>
+  <si>
+    <t>allergies</t>
+  </si>
+  <si>
+    <t>foodPreference</t>
+  </si>
+  <si>
+    <t>cuisineCategory</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>john@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -189,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -198,6 +345,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -765,4 +913,291 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDEF9F35-5020-874F-BB25-D3E9BA50B8F7}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0AEB590-56AA-C04A-B69B-F5C274484CDE}">
+  <dimension ref="A1:A32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC03035-8BC9-954E-8E01-C9E4324E4440}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5">
+        <v>9876543210</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="4">
+        <v>33003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>